<commit_message>
feat: enhance UploadZone component with file validation and loading state; update sample data generation
</commit_message>
<xml_diff>
--- a/backend/input/clientes.xlsx
+++ b/backend/input/clientes.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,12 +442,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Idade</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Cidade</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Valor</t>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
         </is>
       </c>
     </row>
@@ -457,16 +462,21 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ana</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+          <t>Ana Silva</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D2" t="inlineStr">
         <is>
           <t>São Paulo</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>1500.5</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ana@email.com</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -475,16 +485,21 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>João</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Campinas</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>2300</v>
+          <t>João Santos</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>31</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Rio de Janeiro</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>joao@email.com</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -493,16 +508,21 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Maria</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Santos</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>980.25</v>
+          <t>Maria Oliveira</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>28</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>maria@email.com</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -511,16 +531,21 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Carlos</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Sorocaba</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>4100.75</v>
+          <t>Carlos Souza</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>45</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Belo Horizonte</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>carlos@email.com</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -529,16 +554,44 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fernanda</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Osasco</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>1890</v>
+          <t>Beatriz Lima</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>22</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>beatriz@email.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Beatriz Lima</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>22</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>São Paulo</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>beatriz@email.com</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -552,13 +605,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Pedido</t>
+          <t>ID Venda</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -568,60 +621,103 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Quantidade</t>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>101</v>
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ana</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>2</v>
+          <t>Ana Silva</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Notebook</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>4500</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>102</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>João</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>5</v>
+          <t>João Santos</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>103</v>
+        <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Maria</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
+          <t>Maria Oliveira</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Teclado</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>104</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Carlos</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>3</v>
+          <t>Carlos Souza</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Monitor</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Beatriz Lima</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Headset</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>450</v>
       </c>
     </row>
   </sheetData>

</xml_diff>